<commit_message>
Load Hapke Excel metadata rows and select endmembers for unmixing
Parse spectrum ID, grain size, density, and n from Excel rows 2–5 with
REFF from row 6 onward; prefill the parameter panel (lab i/e default
30°/0°); only checked endmembers are kept for single-spectrum and
image Hapke unmixing. Refresh the shipped template and docs.

Co-authored-by: linhoml <linhoml@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/libraries/hapke_endmembers_template.xlsx
+++ b/data/libraries/hapke_endmembers_template.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D162"/>
+  <dimension ref="A1:D166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>wavelength_um</t>
+          <t>mineral / wavelength</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -439,2256 +439,2326 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0.300000188206016</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.55</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>光谱ID</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>OL-01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PX-01</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>PL-01</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>1.01</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>平均粒径_um</t>
+        </is>
       </c>
       <c r="B3" t="n">
-        <v>0.3519629907879534</v>
+        <v>50</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3000002506198358</v>
+        <v>40</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5498000000000001</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>1.02</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>密度_g_cm3</t>
+        </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3539229547863922</v>
+        <v>3.32</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3000003326654042</v>
+        <v>3.5</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5496000000000001</v>
+        <v>2.69</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>1.03</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>折射率_n</t>
+        </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3558768698728919</v>
+        <v>1.69</v>
       </c>
       <c r="C5" t="n">
-        <v>0.3000004401595138</v>
+        <v>1.7</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5494</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1.04</v>
+        <v>1</v>
       </c>
       <c r="B6" t="n">
-        <v>0.3578217232520115</v>
+        <v>0.35</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3000005805275114</v>
+        <v>0.300000188206016</v>
       </c>
       <c r="D6" t="n">
-        <v>0.5492</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1.05</v>
+        <v>1.01</v>
       </c>
       <c r="B7" t="n">
-        <v>0.3597545161008064</v>
+        <v>0.3519629907879534</v>
       </c>
       <c r="C7" t="n">
-        <v>0.3000007632130298</v>
+        <v>0.3000002506198358</v>
       </c>
       <c r="D7" t="n">
-        <v>0.549</v>
+        <v>0.5498000000000001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1.06</v>
+        <v>1.02</v>
       </c>
       <c r="B8" t="n">
-        <v>0.3616722681927952</v>
+        <v>0.3539229547863922</v>
       </c>
       <c r="C8" t="n">
-        <v>0.3000010001819302</v>
+        <v>0.3000003326654042</v>
       </c>
       <c r="D8" t="n">
-        <v>0.5488000000000001</v>
+        <v>0.5496000000000001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1.07</v>
+        <v>1.03</v>
       </c>
       <c r="B9" t="n">
-        <v>0.3635720224932537</v>
+        <v>0.3558768698728919</v>
       </c>
       <c r="C9" t="n">
-        <v>0.3000013065393363</v>
+        <v>0.3000004401595138</v>
       </c>
       <c r="D9" t="n">
-        <v>0.5486000000000001</v>
+        <v>0.5494</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1.08</v>
+        <v>1.04</v>
       </c>
       <c r="B10" t="n">
-        <v>0.3654508497187474</v>
+        <v>0.3578217232520115</v>
       </c>
       <c r="C10" t="n">
-        <v>0.3000017012817093</v>
+        <v>0.3000005805275114</v>
       </c>
       <c r="D10" t="n">
-        <v>0.5484</v>
+        <v>0.5492</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1.09</v>
+        <v>1.05</v>
       </c>
       <c r="B11" t="n">
-        <v>0.3673058528538746</v>
+        <v>0.3597545161008064</v>
       </c>
       <c r="C11" t="n">
-        <v>0.3000022082092957</v>
+        <v>0.3000007632130298</v>
       </c>
       <c r="D11" t="n">
-        <v>0.5482</v>
+        <v>0.549</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1.1</v>
+        <v>1.06</v>
       </c>
       <c r="B12" t="n">
-        <v>0.3691341716182545</v>
+        <v>0.3616722681927952</v>
       </c>
       <c r="C12" t="n">
-        <v>0.3000028570279713</v>
+        <v>0.3000010001819302</v>
       </c>
       <c r="D12" t="n">
-        <v>0.548</v>
+        <v>0.5488000000000001</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1.11</v>
+        <v>1.07</v>
       </c>
       <c r="B13" t="n">
-        <v>0.3709329868768714</v>
+        <v>0.3635720224932537</v>
       </c>
       <c r="C13" t="n">
-        <v>0.3000036846734793</v>
+        <v>0.3000013065393363</v>
       </c>
       <c r="D13" t="n">
-        <v>0.5478000000000001</v>
+        <v>0.5486000000000001</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1.12</v>
+        <v>1.08</v>
       </c>
       <c r="B14" t="n">
-        <v>0.3726995249869773</v>
+        <v>0.3654508497187474</v>
       </c>
       <c r="C14" t="n">
-        <v>0.3000047368952647</v>
+        <v>0.3000017012817093</v>
       </c>
       <c r="D14" t="n">
-        <v>0.5476000000000001</v>
+        <v>0.5484</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1.13</v>
+        <v>1.09</v>
       </c>
       <c r="B15" t="n">
-        <v>0.3744310620748477</v>
+        <v>0.3673058528538746</v>
       </c>
       <c r="C15" t="n">
-        <v>0.3000060701414847</v>
+        <v>0.3000022082092957</v>
       </c>
       <c r="D15" t="n">
-        <v>0.5474</v>
+        <v>0.5482</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1.14</v>
+        <v>1.1</v>
       </c>
       <c r="B16" t="n">
-        <v>0.3761249282357975</v>
+        <v>0.3691341716182545</v>
       </c>
       <c r="C16" t="n">
-        <v>0.3000077537912217</v>
+        <v>0.3000028570279713</v>
       </c>
       <c r="D16" t="n">
-        <v>0.5472</v>
+        <v>0.548</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1.15</v>
+        <v>1.11</v>
       </c>
       <c r="B17" t="n">
-        <v>0.3777785116509801</v>
+        <v>0.3709329868768714</v>
       </c>
       <c r="C17" t="n">
-        <v>0.3000098727843269</v>
+        <v>0.3000036846734793</v>
       </c>
       <c r="D17" t="n">
-        <v>0.547</v>
+        <v>0.5478000000000001</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1.16</v>
+        <v>1.12</v>
       </c>
       <c r="B18" t="n">
-        <v>0.3793892626146236</v>
+        <v>0.3726995249869773</v>
       </c>
       <c r="C18" t="n">
-        <v>0.3000125307035134</v>
+        <v>0.3000047368952647</v>
       </c>
       <c r="D18" t="n">
-        <v>0.5468000000000001</v>
+        <v>0.5476000000000001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1.17</v>
+        <v>1.13</v>
       </c>
       <c r="B19" t="n">
-        <v>0.3809546974654917</v>
+        <v>0.3744310620748477</v>
       </c>
       <c r="C19" t="n">
-        <v>0.3000158533671089</v>
+        <v>0.3000060701414847</v>
       </c>
       <c r="D19" t="n">
-        <v>0.5466000000000001</v>
+        <v>0.5474</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="B20" t="n">
-        <v>0.3824724024165092</v>
+        <v>0.3761249282357975</v>
       </c>
       <c r="C20" t="n">
-        <v>0.3000199929940294</v>
+        <v>0.3000077537912217</v>
       </c>
       <c r="D20" t="n">
-        <v>0.5464</v>
+        <v>0.5472</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1.19</v>
+        <v>1.15</v>
       </c>
       <c r="B21" t="n">
-        <v>0.3839400372766471</v>
+        <v>0.3777785116509801</v>
       </c>
       <c r="C21" t="n">
-        <v>0.3000251330047752</v>
+        <v>0.3000098727843269</v>
       </c>
       <c r="D21" t="n">
-        <v>0.5462</v>
+        <v>0.547</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1.2</v>
+        <v>1.16</v>
       </c>
       <c r="B22" t="n">
-        <v>0.3853553390593274</v>
+        <v>0.3793892626146236</v>
       </c>
       <c r="C22" t="n">
-        <v>0.3000314935232524</v>
+        <v>0.3000125307035134</v>
       </c>
       <c r="D22" t="n">
-        <v>0.546</v>
+        <v>0.5468000000000001</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1.21</v>
+        <v>1.17</v>
       </c>
       <c r="B23" t="n">
-        <v>0.3867161254717843</v>
+        <v>0.3809546974654917</v>
       </c>
       <c r="C23" t="n">
-        <v>0.3000393376436319</v>
+        <v>0.3000158533671089</v>
       </c>
       <c r="D23" t="n">
-        <v>0.5458000000000001</v>
+        <v>0.5466000000000001</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="B24" t="n">
-        <v>0.3880202982800016</v>
+        <v>0.3824724024165092</v>
       </c>
       <c r="C24" t="n">
-        <v>0.3000489785238695</v>
+        <v>0.3000199929940294</v>
       </c>
       <c r="D24" t="n">
-        <v>0.5456000000000001</v>
+        <v>0.5464</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1.23</v>
+        <v>1.19</v>
       </c>
       <c r="B25" t="n">
-        <v>0.3892658465440372</v>
+        <v>0.3839400372766471</v>
       </c>
       <c r="C25" t="n">
-        <v>0.3000607873624943</v>
+        <v>0.3000251330047752</v>
       </c>
       <c r="D25" t="n">
-        <v>0.5454</v>
+        <v>0.5462</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>1.24</v>
+        <v>1.2</v>
       </c>
       <c r="B26" t="n">
-        <v>0.3904508497187474</v>
+        <v>0.3853553390593274</v>
       </c>
       <c r="C26" t="n">
-        <v>0.3000752023073744</v>
+        <v>0.3000314935232524</v>
       </c>
       <c r="D26" t="n">
-        <v>0.5452</v>
+        <v>0.546</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1.25</v>
+        <v>1.21</v>
       </c>
       <c r="B27" t="n">
-        <v>0.3915734806151273</v>
+        <v>0.3867161254717843</v>
       </c>
       <c r="C27" t="n">
-        <v>0.3000927383339124</v>
+        <v>0.3000393376436319</v>
       </c>
       <c r="D27" t="n">
-        <v>0.545</v>
+        <v>0.5458000000000001</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>1.26</v>
+        <v>1.22</v>
       </c>
       <c r="B28" t="n">
-        <v>0.3926320082177046</v>
+        <v>0.3880202982800016</v>
       </c>
       <c r="C28" t="n">
-        <v>0.3001139981150554</v>
+        <v>0.3000489785238695</v>
       </c>
       <c r="D28" t="n">
-        <v>0.5448000000000001</v>
+        <v>0.5456000000000001</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1.27</v>
+        <v>1.23</v>
       </c>
       <c r="B29" t="n">
-        <v>0.3936248003536398</v>
+        <v>0.3892658465440372</v>
       </c>
       <c r="C29" t="n">
-        <v>0.3001396838861702</v>
+        <v>0.3000607873624943</v>
       </c>
       <c r="D29" t="n">
-        <v>0.5446000000000001</v>
+        <v>0.5454</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>1.28</v>
+        <v>1.24</v>
       </c>
       <c r="B30" t="n">
-        <v>0.3945503262094184</v>
+        <v>0.3904508497187474</v>
       </c>
       <c r="C30" t="n">
-        <v>0.3001706102838388</v>
+        <v>0.3000752023073744</v>
       </c>
       <c r="D30" t="n">
-        <v>0.5444</v>
+        <v>0.5452</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>1.29</v>
+        <v>1.25</v>
       </c>
       <c r="B31" t="n">
-        <v>0.3954071586912541</v>
+        <v>0.3915734806151273</v>
       </c>
       <c r="C31" t="n">
-        <v>0.3002077181086515</v>
+        <v>0.3000927383339124</v>
       </c>
       <c r="D31" t="n">
-        <v>0.5442</v>
+        <v>0.545</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>1.3</v>
+        <v>1.26</v>
       </c>
       <c r="B32" t="n">
-        <v>0.3961939766255643</v>
+        <v>0.3926320082177046</v>
       </c>
       <c r="C32" t="n">
-        <v>0.3002520889278755</v>
+        <v>0.3001139981150554</v>
       </c>
       <c r="D32" t="n">
-        <v>0.544</v>
+        <v>0.5448000000000001</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>1.31</v>
+        <v>1.27</v>
       </c>
       <c r="B33" t="n">
-        <v>0.3969095667961242</v>
+        <v>0.3936248003536398</v>
       </c>
       <c r="C33" t="n">
-        <v>0.3003049603943715</v>
+        <v>0.3001396838861702</v>
       </c>
       <c r="D33" t="n">
-        <v>0.5438000000000001</v>
+        <v>0.5446000000000001</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>1.32</v>
+        <v>1.28</v>
       </c>
       <c r="B34" t="n">
-        <v>0.3975528258147577</v>
+        <v>0.3945503262094184</v>
       </c>
       <c r="C34" t="n">
-        <v>0.3003677421133822</v>
+        <v>0.3001706102838388</v>
       </c>
       <c r="D34" t="n">
-        <v>0.5436000000000001</v>
+        <v>0.5444</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>1.33</v>
+        <v>1.29</v>
       </c>
       <c r="B35" t="n">
-        <v>0.3981227618226824</v>
+        <v>0.3954071586912541</v>
       </c>
       <c r="C35" t="n">
-        <v>0.3004420318391043</v>
+        <v>0.3002077181086515</v>
       </c>
       <c r="D35" t="n">
-        <v>0.5434</v>
+        <v>0.5442</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>1.34</v>
+        <v>1.3</v>
       </c>
       <c r="B36" t="n">
-        <v>0.3986184960198838</v>
+        <v>0.3961939766255643</v>
       </c>
       <c r="C36" t="n">
-        <v>0.3005296317287744</v>
+        <v>0.3002520889278755</v>
       </c>
       <c r="D36" t="n">
-        <v>0.5432</v>
+        <v>0.544</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>1.35</v>
+        <v>1.31</v>
       </c>
       <c r="B37" t="n">
-        <v>0.3990392640201615</v>
+        <v>0.3969095667961242</v>
       </c>
       <c r="C37" t="n">
-        <v>0.3006325643241275</v>
+        <v>0.3003049603943715</v>
       </c>
       <c r="D37" t="n">
-        <v>0.543</v>
+        <v>0.5438000000000001</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>1.36</v>
+        <v>1.32</v>
       </c>
       <c r="B38" t="n">
-        <v>0.3993844170297569</v>
+        <v>0.3975528258147577</v>
       </c>
       <c r="C38" t="n">
-        <v>0.3007530878695761</v>
+        <v>0.3003677421133822</v>
       </c>
       <c r="D38" t="n">
-        <v>0.5428000000000001</v>
+        <v>0.5436000000000001</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>1.37</v>
+        <v>1.33</v>
       </c>
       <c r="B39" t="n">
-        <v>0.3996534228477463</v>
+        <v>0.3981227618226824</v>
       </c>
       <c r="C39" t="n">
-        <v>0.3008937105146824</v>
+        <v>0.3004420318391043</v>
       </c>
       <c r="D39" t="n">
-        <v>0.5426000000000001</v>
+        <v>0.5434</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>1.38</v>
+        <v>1.34</v>
       </c>
       <c r="B40" t="n">
-        <v>0.3998458666866564</v>
+        <v>0.3986184960198838</v>
       </c>
       <c r="C40" t="n">
-        <v>0.3010572028871388</v>
+        <v>0.3005296317287744</v>
       </c>
       <c r="D40" t="n">
-        <v>0.5424</v>
+        <v>0.5432</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>1.39</v>
+        <v>1.35</v>
       </c>
       <c r="B41" t="n">
-        <v>0.3999614518120361</v>
+        <v>0.3990392640201615</v>
       </c>
       <c r="C41" t="n">
-        <v>0.3012466084635468</v>
+        <v>0.3006325643241275</v>
       </c>
       <c r="D41" t="n">
-        <v>0.5422</v>
+        <v>0.543</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="B42" t="n">
-        <v>0.4</v>
+        <v>0.3993844170297569</v>
       </c>
       <c r="C42" t="n">
-        <v>0.3014652511110987</v>
+        <v>0.3007530878695761</v>
       </c>
       <c r="D42" t="n">
-        <v>0.542</v>
+        <v>0.5428000000000001</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>1.41</v>
+        <v>1.37</v>
       </c>
       <c r="B43" t="n">
-        <v>0.3999614518120361</v>
+        <v>0.3996534228477463</v>
       </c>
       <c r="C43" t="n">
-        <v>0.3017167391264065</v>
+        <v>0.3008937105146824</v>
       </c>
       <c r="D43" t="n">
-        <v>0.5418000000000001</v>
+        <v>0.5426000000000001</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>1.42</v>
+        <v>1.38</v>
       </c>
       <c r="B44" t="n">
         <v>0.3998458666866564</v>
       </c>
       <c r="C44" t="n">
-        <v>0.3020049650610047</v>
+        <v>0.3010572028871388</v>
       </c>
       <c r="D44" t="n">
-        <v>0.5416000000000001</v>
+        <v>0.5424</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>1.43</v>
+        <v>1.39</v>
       </c>
       <c r="B45" t="n">
-        <v>0.3996534228477463</v>
+        <v>0.3999614518120361</v>
       </c>
       <c r="C45" t="n">
-        <v>0.3023341005994574</v>
+        <v>0.3012466084635468</v>
       </c>
       <c r="D45" t="n">
-        <v>0.5414</v>
+        <v>0.5422</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>1.44</v>
+        <v>1.4</v>
       </c>
       <c r="B46" t="n">
-        <v>0.3993844170297569</v>
+        <v>0.4</v>
       </c>
       <c r="C46" t="n">
-        <v>0.3027085857485619</v>
+        <v>0.3014652511110987</v>
       </c>
       <c r="D46" t="n">
-        <v>0.5412</v>
+        <v>0.542</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>1.45</v>
+        <v>1.41</v>
       </c>
       <c r="B47" t="n">
-        <v>0.3990392640201615</v>
+        <v>0.3999614518120361</v>
       </c>
       <c r="C47" t="n">
-        <v>0.303133111607919</v>
+        <v>0.3017167391264065</v>
       </c>
       <c r="D47" t="n">
-        <v>0.541</v>
+        <v>0.5418000000000001</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>1.46</v>
+        <v>1.42</v>
       </c>
       <c r="B48" t="n">
-        <v>0.3986184960198838</v>
+        <v>0.3998458666866564</v>
       </c>
       <c r="C48" t="n">
-        <v>0.3036125960259889</v>
+        <v>0.3020049650610047</v>
       </c>
       <c r="D48" t="n">
-        <v>0.5408000000000001</v>
+        <v>0.5416000000000001</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>1.47</v>
+        <v>1.43</v>
       </c>
       <c r="B49" t="n">
-        <v>0.3981227618226823</v>
+        <v>0.3996534228477463</v>
       </c>
       <c r="C49" t="n">
-        <v>0.3041521515043045</v>
+        <v>0.3023341005994574</v>
       </c>
       <c r="D49" t="n">
-        <v>0.5406000000000001</v>
+        <v>0.5414</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>1.48</v>
+        <v>1.44</v>
       </c>
       <c r="B50" t="n">
-        <v>0.3975528258147576</v>
+        <v>0.3993844170297569</v>
       </c>
       <c r="C50" t="n">
-        <v>0.3047570447979443</v>
+        <v>0.3027085857485619</v>
       </c>
       <c r="D50" t="n">
-        <v>0.5404</v>
+        <v>0.5412</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>1.49</v>
+        <v>1.45</v>
       </c>
       <c r="B51" t="n">
-        <v>0.3969095667961242</v>
+        <v>0.3990392640201615</v>
       </c>
       <c r="C51" t="n">
-        <v>0.3054326477742968</v>
+        <v>0.303133111607919</v>
       </c>
       <c r="D51" t="n">
-        <v>0.5402</v>
+        <v>0.541</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>1.5</v>
+        <v>1.46</v>
       </c>
       <c r="B52" t="n">
-        <v>0.3961939766255643</v>
+        <v>0.3986184960198838</v>
       </c>
       <c r="C52" t="n">
-        <v>0.306184379235464</v>
+        <v>0.3036125960259889</v>
       </c>
       <c r="D52" t="n">
-        <v>0.54</v>
+        <v>0.5408000000000001</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>1.51</v>
+        <v>1.47</v>
       </c>
       <c r="B53" t="n">
-        <v>0.395407158691254</v>
+        <v>0.3981227618226823</v>
       </c>
       <c r="C53" t="n">
-        <v>0.3070176375823834</v>
+        <v>0.3041521515043045</v>
       </c>
       <c r="D53" t="n">
-        <v>0.5398000000000001</v>
+        <v>0.5406000000000001</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>1.52</v>
+        <v>1.48</v>
       </c>
       <c r="B54" t="n">
-        <v>0.3945503262094183</v>
+        <v>0.3975528258147576</v>
       </c>
       <c r="C54" t="n">
-        <v>0.3079377243999091</v>
+        <v>0.3047570447979443</v>
       </c>
       <c r="D54" t="n">
-        <v>0.5396000000000001</v>
+        <v>0.5404</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>1.53</v>
+        <v>1.49</v>
       </c>
       <c r="B55" t="n">
-        <v>0.3936248003536398</v>
+        <v>0.3969095667961242</v>
       </c>
       <c r="C55" t="n">
-        <v>0.3089497592696023</v>
+        <v>0.3054326477742968</v>
       </c>
       <c r="D55" t="n">
-        <v>0.5394</v>
+        <v>0.5402</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>1.54</v>
+        <v>1.5</v>
       </c>
       <c r="B56" t="n">
-        <v>0.3926320082177046</v>
+        <v>0.3961939766255643</v>
       </c>
       <c r="C56" t="n">
-        <v>0.3100585863675543</v>
+        <v>0.306184379235464</v>
       </c>
       <c r="D56" t="n">
-        <v>0.5392</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>1.55</v>
+        <v>1.51</v>
       </c>
       <c r="B57" t="n">
-        <v>0.3915734806151272</v>
+        <v>0.395407158691254</v>
       </c>
       <c r="C57" t="n">
-        <v>0.3112686736736837</v>
+        <v>0.3070176375823834</v>
       </c>
       <c r="D57" t="n">
-        <v>0.539</v>
+        <v>0.5398000000000001</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>1.56</v>
+        <v>1.52</v>
       </c>
       <c r="B58" t="n">
-        <v>0.3904508497187473</v>
+        <v>0.3945503262094183</v>
       </c>
       <c r="C58" t="n">
-        <v>0.3125840059008644</v>
+        <v>0.3079377243999091</v>
       </c>
       <c r="D58" t="n">
-        <v>0.5388000000000001</v>
+        <v>0.5396000000000001</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>1.570000000000001</v>
+        <v>1.53</v>
       </c>
       <c r="B59" t="n">
-        <v>0.3892658465440372</v>
+        <v>0.3936248003536398</v>
       </c>
       <c r="C59" t="n">
-        <v>0.3140079725400092</v>
+        <v>0.3089497592696023</v>
       </c>
       <c r="D59" t="n">
-        <v>0.5386000000000001</v>
+        <v>0.5394</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>1.580000000000001</v>
+        <v>1.54</v>
       </c>
       <c r="B60" t="n">
-        <v>0.3880202982800015</v>
+        <v>0.3926320082177046</v>
       </c>
       <c r="C60" t="n">
-        <v>0.3155432527028391</v>
+        <v>0.3100585863675543</v>
       </c>
       <c r="D60" t="n">
-        <v>0.5384</v>
+        <v>0.5392</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>1.590000000000001</v>
+        <v>1.55</v>
       </c>
       <c r="B61" t="n">
-        <v>0.3867161254717842</v>
+        <v>0.3915734806151272</v>
       </c>
       <c r="C61" t="n">
-        <v>0.3171916987185766</v>
+        <v>0.3112686736736837</v>
       </c>
       <c r="D61" t="n">
-        <v>0.5382</v>
+        <v>0.539</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>1.600000000000001</v>
+        <v>1.56</v>
       </c>
       <c r="B62" t="n">
-        <v>0.3853553390593273</v>
+        <v>0.3904508497187473</v>
       </c>
       <c r="C62" t="n">
-        <v>0.3189542206945699</v>
+        <v>0.3125840059008644</v>
       </c>
       <c r="D62" t="n">
-        <v>0.538</v>
+        <v>0.5388000000000001</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>1.610000000000001</v>
+        <v>1.570000000000001</v>
       </c>
       <c r="B63" t="n">
-        <v>0.383940037276647</v>
+        <v>0.3892658465440372</v>
       </c>
       <c r="C63" t="n">
-        <v>0.3208306744738424</v>
+        <v>0.3140079725400092</v>
       </c>
       <c r="D63" t="n">
-        <v>0.5378000000000001</v>
+        <v>0.5386000000000001</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>1.620000000000001</v>
+        <v>1.580000000000001</v>
       </c>
       <c r="B64" t="n">
-        <v>0.3824724024165091</v>
+        <v>0.3880202982800015</v>
       </c>
       <c r="C64" t="n">
-        <v>0.3228197556045845</v>
+        <v>0.3155432527028391</v>
       </c>
       <c r="D64" t="n">
-        <v>0.5376000000000001</v>
+        <v>0.5384</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>1.630000000000001</v>
+        <v>1.590000000000001</v>
       </c>
       <c r="B65" t="n">
-        <v>0.3809546974654916</v>
+        <v>0.3867161254717842</v>
       </c>
       <c r="C65" t="n">
-        <v>0.3249189020677927</v>
+        <v>0.3171916987185766</v>
       </c>
       <c r="D65" t="n">
-        <v>0.5374</v>
+        <v>0.5382</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>1.640000000000001</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="B66" t="n">
-        <v>0.3793892626146235</v>
+        <v>0.3853553390593273</v>
       </c>
       <c r="C66" t="n">
-        <v>0.3271242085803555</v>
+        <v>0.3189542206945699</v>
       </c>
       <c r="D66" t="n">
-        <v>0.5372</v>
+        <v>0.538</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>1.650000000000001</v>
+        <v>1.610000000000001</v>
       </c>
       <c r="B67" t="n">
-        <v>0.37777851165098</v>
+        <v>0.383940037276647</v>
       </c>
       <c r="C67" t="n">
-        <v>0.3294303552937156</v>
+        <v>0.3208306744738424</v>
       </c>
       <c r="D67" t="n">
-        <v>0.537</v>
+        <v>0.5378000000000001</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>1.660000000000001</v>
+        <v>1.620000000000001</v>
       </c>
       <c r="B68" t="n">
-        <v>0.3761249282357974</v>
+        <v>0.3824724024165091</v>
       </c>
       <c r="C68" t="n">
-        <v>0.3318305536360965</v>
+        <v>0.3228197556045845</v>
       </c>
       <c r="D68" t="n">
-        <v>0.5368000000000001</v>
+        <v>0.5376000000000001</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>1.670000000000001</v>
+        <v>1.630000000000001</v>
       </c>
       <c r="B69" t="n">
-        <v>0.3744310620748477</v>
+        <v>0.3809546974654916</v>
       </c>
       <c r="C69" t="n">
-        <v>0.334316511894326</v>
+        <v>0.3249189020677927</v>
       </c>
       <c r="D69" t="n">
-        <v>0.5366000000000001</v>
+        <v>0.5374</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>1.680000000000001</v>
+        <v>1.640000000000001</v>
       </c>
       <c r="B70" t="n">
-        <v>0.3726995249869772</v>
+        <v>0.3793892626146235</v>
       </c>
       <c r="C70" t="n">
-        <v>0.3368784228968669</v>
+        <v>0.3271242085803555</v>
       </c>
       <c r="D70" t="n">
-        <v>0.5364</v>
+        <v>0.5372</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>1.690000000000001</v>
+        <v>1.650000000000001</v>
       </c>
       <c r="B71" t="n">
-        <v>0.3709329868768713</v>
+        <v>0.37777851165098</v>
       </c>
       <c r="C71" t="n">
-        <v>0.3395049758426679</v>
+        <v>0.3294303552937156</v>
       </c>
       <c r="D71" t="n">
-        <v>0.5362</v>
+        <v>0.537</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>1.700000000000001</v>
+        <v>1.660000000000001</v>
       </c>
       <c r="B72" t="n">
-        <v>0.3691341716182543</v>
+        <v>0.3761249282357974</v>
       </c>
       <c r="C72" t="n">
-        <v>0.342183393923444</v>
+        <v>0.3318305536360965</v>
       </c>
       <c r="D72" t="n">
-        <v>0.536</v>
+        <v>0.5368000000000001</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>1.710000000000001</v>
+        <v>1.670000000000001</v>
       </c>
       <c r="B73" t="n">
-        <v>0.3673058528538745</v>
+        <v>0.3744310620748477</v>
       </c>
       <c r="C73" t="n">
-        <v>0.344899498915459</v>
+        <v>0.334316511894326</v>
       </c>
       <c r="D73" t="n">
-        <v>0.5358000000000001</v>
+        <v>0.5366000000000001</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>1.720000000000001</v>
+        <v>1.680000000000001</v>
       </c>
       <c r="B74" t="n">
-        <v>0.3654508497187473</v>
+        <v>0.3726995249869772</v>
       </c>
       <c r="C74" t="n">
-        <v>0.3476378033791418</v>
+        <v>0.3368784228968669</v>
       </c>
       <c r="D74" t="n">
-        <v>0.5356000000000001</v>
+        <v>0.5364</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>1.730000000000001</v>
+        <v>1.690000000000001</v>
       </c>
       <c r="B75" t="n">
-        <v>0.3635720224932536</v>
+        <v>0.3709329868768713</v>
       </c>
       <c r="C75" t="n">
-        <v>0.3503816305120804</v>
+        <v>0.3395049758426679</v>
       </c>
       <c r="D75" t="n">
-        <v>0.5354</v>
+        <v>0.5362</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>1.740000000000001</v>
+        <v>1.700000000000001</v>
       </c>
       <c r="B76" t="n">
-        <v>0.3616722681927951</v>
+        <v>0.3691341716182543</v>
       </c>
       <c r="C76" t="n">
-        <v>0.353113261066838</v>
+        <v>0.342183393923444</v>
       </c>
       <c r="D76" t="n">
-        <v>0.5352</v>
+        <v>0.536</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>1.750000000000001</v>
+        <v>1.710000000000001</v>
       </c>
       <c r="B77" t="n">
-        <v>0.3597545161008063</v>
+        <v>0.3673058528538745</v>
       </c>
       <c r="C77" t="n">
-        <v>0.3558141060856826</v>
+        <v>0.344899498915459</v>
       </c>
       <c r="D77" t="n">
-        <v>0.535</v>
+        <v>0.5358000000000001</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>1.760000000000001</v>
+        <v>1.720000000000001</v>
       </c>
       <c r="B78" t="n">
-        <v>0.3578217232520114</v>
+        <v>0.3654508497187473</v>
       </c>
       <c r="C78" t="n">
-        <v>0.3584649035376005</v>
+        <v>0.3476378033791418</v>
       </c>
       <c r="D78" t="n">
-        <v>0.5348000000000001</v>
+        <v>0.5356000000000001</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>1.770000000000001</v>
+        <v>1.730000000000001</v>
       </c>
       <c r="B79" t="n">
-        <v>0.3558768698728917</v>
+        <v>0.3635720224932536</v>
       </c>
       <c r="C79" t="n">
-        <v>0.361045936288107</v>
+        <v>0.3503816305120804</v>
       </c>
       <c r="D79" t="n">
-        <v>0.5346000000000001</v>
+        <v>0.5354</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>1.780000000000001</v>
+        <v>1.740000000000001</v>
       </c>
       <c r="B80" t="n">
-        <v>0.3539229547863921</v>
+        <v>0.3616722681927951</v>
       </c>
       <c r="C80" t="n">
-        <v>0.3635372682093239</v>
+        <v>0.353113261066838</v>
       </c>
       <c r="D80" t="n">
-        <v>0.5344</v>
+        <v>0.5352</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>1.790000000000001</v>
+        <v>1.750000000000001</v>
       </c>
       <c r="B81" t="n">
-        <v>0.3519629907879533</v>
+        <v>0.3597545161008063</v>
       </c>
       <c r="C81" t="n">
-        <v>0.3659189946665364</v>
+        <v>0.3558141060856826</v>
       </c>
       <c r="D81" t="n">
-        <v>0.5342</v>
+        <v>0.535</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>1.800000000000001</v>
+        <v>1.760000000000001</v>
       </c>
       <c r="B82" t="n">
-        <v>0.3499999999999999</v>
+        <v>0.3578217232520114</v>
       </c>
       <c r="C82" t="n">
-        <v>0.3681715031172971</v>
+        <v>0.3584649035376005</v>
       </c>
       <c r="D82" t="n">
-        <v>0.534</v>
+        <v>0.5348000000000001</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>1.810000000000001</v>
+        <v>1.770000000000001</v>
       </c>
       <c r="B83" t="n">
-        <v>0.3480370092120464</v>
+        <v>0.3558768698728917</v>
       </c>
       <c r="C83" t="n">
-        <v>0.3702757391479947</v>
+        <v>0.361045936288107</v>
       </c>
       <c r="D83" t="n">
-        <v>0.5338000000000001</v>
+        <v>0.5346000000000001</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>1.820000000000001</v>
+        <v>1.780000000000001</v>
       </c>
       <c r="B84" t="n">
-        <v>0.3460770452136076</v>
+        <v>0.3539229547863921</v>
       </c>
       <c r="C84" t="n">
-        <v>0.3722134729664755</v>
+        <v>0.3635372682093239</v>
       </c>
       <c r="D84" t="n">
-        <v>0.5336000000000001</v>
+        <v>0.5344</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>1.830000000000001</v>
+        <v>1.790000000000001</v>
       </c>
       <c r="B85" t="n">
-        <v>0.344123130127108</v>
+        <v>0.3519629907879533</v>
       </c>
       <c r="C85" t="n">
-        <v>0.373967561180817</v>
+        <v>0.3659189946665364</v>
       </c>
       <c r="D85" t="n">
-        <v>0.5334</v>
+        <v>0.5342</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>1.840000000000001</v>
+        <v>1.800000000000001</v>
       </c>
       <c r="B86" t="n">
-        <v>0.3421782767479883</v>
+        <v>0.3499999999999999</v>
       </c>
       <c r="C86" t="n">
-        <v>0.375522198633427</v>
+        <v>0.3681715031172971</v>
       </c>
       <c r="D86" t="n">
-        <v>0.5332</v>
+        <v>0.534</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>1.850000000000001</v>
+        <v>1.810000000000001</v>
       </c>
       <c r="B87" t="n">
-        <v>0.3402454838991935</v>
+        <v>0.3480370092120464</v>
       </c>
       <c r="C87" t="n">
-        <v>0.3768631551321859</v>
+        <v>0.3702757391479947</v>
       </c>
       <c r="D87" t="n">
-        <v>0.533</v>
+        <v>0.5338000000000001</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>1.860000000000001</v>
+        <v>1.820000000000001</v>
       </c>
       <c r="B88" t="n">
-        <v>0.3383277318072045</v>
+        <v>0.3460770452136076</v>
       </c>
       <c r="C88" t="n">
-        <v>0.3779779921281436</v>
+        <v>0.3722134729664755</v>
       </c>
       <c r="D88" t="n">
-        <v>0.5328000000000001</v>
+        <v>0.5336000000000001</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>1.870000000000001</v>
+        <v>1.830000000000001</v>
       </c>
       <c r="B89" t="n">
-        <v>0.3364279775067461</v>
+        <v>0.344123130127108</v>
       </c>
       <c r="C89" t="n">
-        <v>0.3788562547297955</v>
+        <v>0.373967561180817</v>
       </c>
       <c r="D89" t="n">
-        <v>0.5326000000000001</v>
+        <v>0.5334</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>1.880000000000001</v>
+        <v>1.840000000000001</v>
       </c>
       <c r="B90" t="n">
-        <v>0.3345491502812525</v>
+        <v>0.3421782767479883</v>
       </c>
       <c r="C90" t="n">
-        <v>0.3794896349103319</v>
+        <v>0.375522198633427</v>
       </c>
       <c r="D90" t="n">
-        <v>0.5324</v>
+        <v>0.5332</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>1.890000000000001</v>
+        <v>1.850000000000001</v>
       </c>
       <c r="B91" t="n">
-        <v>0.3326941471461252</v>
+        <v>0.3402454838991935</v>
       </c>
       <c r="C91" t="n">
-        <v>0.3798721023454085</v>
+        <v>0.3768631551321859</v>
       </c>
       <c r="D91" t="n">
-        <v>0.5322</v>
+        <v>0.533</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>1.900000000000001</v>
+        <v>1.860000000000001</v>
       </c>
       <c r="B92" t="n">
-        <v>0.3308658283817453</v>
+        <v>0.3383277318072045</v>
       </c>
       <c r="C92" t="n">
-        <v>0.38</v>
+        <v>0.3779779921281436</v>
       </c>
       <c r="D92" t="n">
-        <v>0.532</v>
+        <v>0.5328000000000001</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>1.910000000000001</v>
+        <v>1.870000000000001</v>
       </c>
       <c r="B93" t="n">
-        <v>0.3290670131231285</v>
+        <v>0.3364279775067461</v>
       </c>
       <c r="C93" t="n">
-        <v>0.3798721023454085</v>
+        <v>0.3788562547297955</v>
       </c>
       <c r="D93" t="n">
-        <v>0.5318000000000001</v>
+        <v>0.5326000000000001</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>1.920000000000001</v>
+        <v>1.880000000000001</v>
       </c>
       <c r="B94" t="n">
-        <v>0.3273004750130225</v>
+        <v>0.3345491502812525</v>
       </c>
       <c r="C94" t="n">
         <v>0.3794896349103319</v>
       </c>
       <c r="D94" t="n">
-        <v>0.5316000000000001</v>
+        <v>0.5324</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>1.930000000000001</v>
+        <v>1.890000000000001</v>
       </c>
       <c r="B95" t="n">
-        <v>0.3255689379251521</v>
+        <v>0.3326941471461252</v>
       </c>
       <c r="C95" t="n">
-        <v>0.3788562547297953</v>
+        <v>0.3798721023454085</v>
       </c>
       <c r="D95" t="n">
-        <v>0.5314</v>
+        <v>0.5322</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>1.940000000000001</v>
+        <v>1.900000000000001</v>
       </c>
       <c r="B96" t="n">
-        <v>0.3238750717642024</v>
+        <v>0.3308658283817453</v>
       </c>
       <c r="C96" t="n">
-        <v>0.3779779921281434</v>
+        <v>0.38</v>
       </c>
       <c r="D96" t="n">
-        <v>0.5312</v>
+        <v>0.532</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>1.950000000000001</v>
+        <v>1.910000000000001</v>
       </c>
       <c r="B97" t="n">
-        <v>0.3222214883490198</v>
+        <v>0.3290670131231285</v>
       </c>
       <c r="C97" t="n">
-        <v>0.3768631551321857</v>
+        <v>0.3798721023454085</v>
       </c>
       <c r="D97" t="n">
-        <v>0.531</v>
+        <v>0.5318000000000001</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>1.960000000000001</v>
+        <v>1.920000000000001</v>
       </c>
       <c r="B98" t="n">
-        <v>0.3206107373853762</v>
+        <v>0.3273004750130225</v>
       </c>
       <c r="C98" t="n">
-        <v>0.3755221986334267</v>
+        <v>0.3794896349103319</v>
       </c>
       <c r="D98" t="n">
-        <v>0.5308</v>
+        <v>0.5316000000000001</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>1.970000000000001</v>
+        <v>1.930000000000001</v>
       </c>
       <c r="B99" t="n">
-        <v>0.3190453025345081</v>
+        <v>0.3255689379251521</v>
       </c>
       <c r="C99" t="n">
-        <v>0.3739675611808167</v>
+        <v>0.3788562547297953</v>
       </c>
       <c r="D99" t="n">
-        <v>0.5306000000000001</v>
+        <v>0.5314</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>1.980000000000001</v>
+        <v>1.940000000000001</v>
       </c>
       <c r="B100" t="n">
-        <v>0.3175275975834907</v>
+        <v>0.3238750717642024</v>
       </c>
       <c r="C100" t="n">
-        <v>0.3722134729664752</v>
+        <v>0.3779779921281434</v>
       </c>
       <c r="D100" t="n">
-        <v>0.5304</v>
+        <v>0.5312</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>1.990000000000001</v>
+        <v>1.950000000000001</v>
       </c>
       <c r="B101" t="n">
-        <v>0.3160599627233528</v>
+        <v>0.3222214883490198</v>
       </c>
       <c r="C101" t="n">
-        <v>0.3702757391479943</v>
+        <v>0.3768631551321857</v>
       </c>
       <c r="D101" t="n">
-        <v>0.5302</v>
+        <v>0.531</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>2.000000000000001</v>
+        <v>1.960000000000001</v>
       </c>
       <c r="B102" t="n">
-        <v>0.3146446609406725</v>
+        <v>0.3206107373853762</v>
       </c>
       <c r="C102" t="n">
-        <v>0.3681715031172967</v>
+        <v>0.3755221986334267</v>
       </c>
       <c r="D102" t="n">
-        <v>0.53</v>
+        <v>0.5308</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>2.010000000000001</v>
+        <v>1.970000000000001</v>
       </c>
       <c r="B103" t="n">
-        <v>0.3132838745282156</v>
+        <v>0.3190453025345081</v>
       </c>
       <c r="C103" t="n">
-        <v>0.3659189946665361</v>
+        <v>0.3739675611808167</v>
       </c>
       <c r="D103" t="n">
-        <v>0.5298</v>
+        <v>0.5306000000000001</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>2.020000000000001</v>
+        <v>1.980000000000001</v>
       </c>
       <c r="B104" t="n">
-        <v>0.3119797017199983</v>
+        <v>0.3175275975834907</v>
       </c>
       <c r="C104" t="n">
-        <v>0.3635372682093235</v>
+        <v>0.3722134729664752</v>
       </c>
       <c r="D104" t="n">
-        <v>0.5296000000000001</v>
+        <v>0.5304</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>2.030000000000001</v>
+        <v>1.990000000000001</v>
       </c>
       <c r="B105" t="n">
-        <v>0.3107341534559626</v>
+        <v>0.3160599627233528</v>
       </c>
       <c r="C105" t="n">
-        <v>0.3610459362881066</v>
+        <v>0.3702757391479943</v>
       </c>
       <c r="D105" t="n">
-        <v>0.5294</v>
+        <v>0.5302</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>2.040000000000001</v>
+        <v>2.000000000000001</v>
       </c>
       <c r="B106" t="n">
-        <v>0.3095491502812525</v>
+        <v>0.3146446609406725</v>
       </c>
       <c r="C106" t="n">
-        <v>0.3584649035376</v>
+        <v>0.3681715031172967</v>
       </c>
       <c r="D106" t="n">
-        <v>0.5292</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>2.050000000000001</v>
+        <v>2.010000000000001</v>
       </c>
       <c r="B107" t="n">
-        <v>0.3084265193848726</v>
+        <v>0.3132838745282156</v>
       </c>
       <c r="C107" t="n">
-        <v>0.3558141060856823</v>
+        <v>0.3659189946665361</v>
       </c>
       <c r="D107" t="n">
-        <v>0.529</v>
+        <v>0.5298</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>2.060000000000001</v>
+        <v>2.020000000000001</v>
       </c>
       <c r="B108" t="n">
-        <v>0.3073679917822953</v>
+        <v>0.3119797017199983</v>
       </c>
       <c r="C108" t="n">
-        <v>0.3531132610668376</v>
+        <v>0.3635372682093235</v>
       </c>
       <c r="D108" t="n">
-        <v>0.5288</v>
+        <v>0.5296000000000001</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>2.070000000000001</v>
+        <v>2.030000000000001</v>
       </c>
       <c r="B109" t="n">
-        <v>0.30637519964636</v>
+        <v>0.3107341534559626</v>
       </c>
       <c r="C109" t="n">
-        <v>0.3503816305120799</v>
+        <v>0.3610459362881066</v>
       </c>
       <c r="D109" t="n">
-        <v>0.5286000000000001</v>
+        <v>0.5294</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>2.080000000000001</v>
+        <v>2.040000000000001</v>
       </c>
       <c r="B110" t="n">
-        <v>0.3054496737905815</v>
+        <v>0.3095491502812525</v>
       </c>
       <c r="C110" t="n">
-        <v>0.3476378033791413</v>
+        <v>0.3584649035376</v>
       </c>
       <c r="D110" t="n">
-        <v>0.5284</v>
+        <v>0.5292</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>2.090000000000001</v>
+        <v>2.050000000000001</v>
       </c>
       <c r="B111" t="n">
-        <v>0.3045928413087459</v>
+        <v>0.3084265193848726</v>
       </c>
       <c r="C111" t="n">
-        <v>0.3448994989154586</v>
+        <v>0.3558141060856823</v>
       </c>
       <c r="D111" t="n">
-        <v>0.5282</v>
+        <v>0.529</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>2.100000000000001</v>
+        <v>2.060000000000001</v>
       </c>
       <c r="B112" t="n">
-        <v>0.3038060233744356</v>
+        <v>0.3073679917822953</v>
       </c>
       <c r="C112" t="n">
-        <v>0.3421833939234436</v>
+        <v>0.3531132610668376</v>
       </c>
       <c r="D112" t="n">
-        <v>0.528</v>
+        <v>0.5288</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>2.110000000000001</v>
+        <v>2.070000000000001</v>
       </c>
       <c r="B113" t="n">
-        <v>0.3030904332038757</v>
+        <v>0.30637519964636</v>
       </c>
       <c r="C113" t="n">
-        <v>0.3395049758426674</v>
+        <v>0.3503816305120799</v>
       </c>
       <c r="D113" t="n">
-        <v>0.5278</v>
+        <v>0.5286000000000001</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>2.120000000000001</v>
+        <v>2.080000000000001</v>
       </c>
       <c r="B114" t="n">
-        <v>0.3024471741852423</v>
+        <v>0.3054496737905815</v>
       </c>
       <c r="C114" t="n">
-        <v>0.3368784228968664</v>
+        <v>0.3476378033791413</v>
       </c>
       <c r="D114" t="n">
-        <v>0.5276000000000001</v>
+        <v>0.5284</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>2.130000000000001</v>
+        <v>2.090000000000001</v>
       </c>
       <c r="B115" t="n">
-        <v>0.3018772381773176</v>
+        <v>0.3045928413087459</v>
       </c>
       <c r="C115" t="n">
-        <v>0.3343165118943256</v>
+        <v>0.3448994989154586</v>
       </c>
       <c r="D115" t="n">
-        <v>0.5274</v>
+        <v>0.5282</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>2.140000000000001</v>
+        <v>2.100000000000001</v>
       </c>
       <c r="B116" t="n">
-        <v>0.3013815039801161</v>
+        <v>0.3038060233744356</v>
       </c>
       <c r="C116" t="n">
-        <v>0.3318305536360961</v>
+        <v>0.3421833939234436</v>
       </c>
       <c r="D116" t="n">
-        <v>0.5272</v>
+        <v>0.528</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>2.150000000000001</v>
+        <v>2.110000000000001</v>
       </c>
       <c r="B117" t="n">
-        <v>0.3009607359798384</v>
+        <v>0.3030904332038757</v>
       </c>
       <c r="C117" t="n">
-        <v>0.3294303552937151</v>
+        <v>0.3395049758426674</v>
       </c>
       <c r="D117" t="n">
-        <v>0.527</v>
+        <v>0.5278</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>2.160000000000001</v>
+        <v>2.120000000000001</v>
       </c>
       <c r="B118" t="n">
-        <v>0.300615582970243</v>
+        <v>0.3024471741852423</v>
       </c>
       <c r="C118" t="n">
-        <v>0.3271242085803551</v>
+        <v>0.3368784228968664</v>
       </c>
       <c r="D118" t="n">
-        <v>0.5268</v>
+        <v>0.5276000000000001</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>2.170000000000001</v>
+        <v>2.130000000000001</v>
       </c>
       <c r="B119" t="n">
-        <v>0.3003465771522537</v>
+        <v>0.3018772381773176</v>
       </c>
       <c r="C119" t="n">
-        <v>0.3249189020677924</v>
+        <v>0.3343165118943256</v>
       </c>
       <c r="D119" t="n">
-        <v>0.5266000000000001</v>
+        <v>0.5274</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>2.180000000000001</v>
+        <v>2.140000000000001</v>
       </c>
       <c r="B120" t="n">
-        <v>0.3001541333133436</v>
+        <v>0.3013815039801161</v>
       </c>
       <c r="C120" t="n">
-        <v>0.3228197556045842</v>
+        <v>0.3318305536360961</v>
       </c>
       <c r="D120" t="n">
-        <v>0.5264</v>
+        <v>0.5272</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>2.190000000000001</v>
+        <v>2.150000000000001</v>
       </c>
       <c r="B121" t="n">
-        <v>0.3000385481879638</v>
+        <v>0.3009607359798384</v>
       </c>
       <c r="C121" t="n">
-        <v>0.3208306744738421</v>
+        <v>0.3294303552937151</v>
       </c>
       <c r="D121" t="n">
-        <v>0.5262</v>
+        <v>0.527</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>2.200000000000001</v>
+        <v>2.160000000000001</v>
       </c>
       <c r="B122" t="n">
-        <v>0.3</v>
+        <v>0.300615582970243</v>
       </c>
       <c r="C122" t="n">
-        <v>0.3189542206945695</v>
+        <v>0.3271242085803551</v>
       </c>
       <c r="D122" t="n">
-        <v>0.526</v>
+        <v>0.5268</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>2.210000000000001</v>
+        <v>2.170000000000001</v>
       </c>
       <c r="B123" t="n">
-        <v>0.3000385481879638</v>
+        <v>0.3003465771522537</v>
       </c>
       <c r="C123" t="n">
-        <v>0.3171916987185763</v>
+        <v>0.3249189020677924</v>
       </c>
       <c r="D123" t="n">
-        <v>0.5258</v>
+        <v>0.5266000000000001</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>2.220000000000001</v>
+        <v>2.180000000000001</v>
       </c>
       <c r="B124" t="n">
         <v>0.3001541333133436</v>
       </c>
       <c r="C124" t="n">
-        <v>0.3155432527028388</v>
+        <v>0.3228197556045842</v>
       </c>
       <c r="D124" t="n">
-        <v>0.5256000000000001</v>
+        <v>0.5264</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>2.230000000000001</v>
+        <v>2.190000000000001</v>
       </c>
       <c r="B125" t="n">
-        <v>0.3003465771522537</v>
+        <v>0.3000385481879638</v>
       </c>
       <c r="C125" t="n">
-        <v>0.3140079725400088</v>
+        <v>0.3208306744738421</v>
       </c>
       <c r="D125" t="n">
-        <v>0.5254</v>
+        <v>0.5262</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>2.240000000000001</v>
+        <v>2.200000000000001</v>
       </c>
       <c r="B126" t="n">
-        <v>0.3006155829702431</v>
+        <v>0.3</v>
       </c>
       <c r="C126" t="n">
-        <v>0.3125840059008641</v>
+        <v>0.3189542206945695</v>
       </c>
       <c r="D126" t="n">
-        <v>0.5252</v>
+        <v>0.526</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>2.250000000000001</v>
+        <v>2.210000000000001</v>
       </c>
       <c r="B127" t="n">
-        <v>0.3009607359798385</v>
+        <v>0.3000385481879638</v>
       </c>
       <c r="C127" t="n">
-        <v>0.3112686736736835</v>
+        <v>0.3171916987185763</v>
       </c>
       <c r="D127" t="n">
-        <v>0.525</v>
+        <v>0.5258</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>2.260000000000001</v>
+        <v>2.220000000000001</v>
       </c>
       <c r="B128" t="n">
-        <v>0.3013815039801162</v>
+        <v>0.3001541333133436</v>
       </c>
       <c r="C128" t="n">
-        <v>0.3100585863675541</v>
+        <v>0.3155432527028388</v>
       </c>
       <c r="D128" t="n">
-        <v>0.5248</v>
+        <v>0.5256000000000001</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>2.270000000000001</v>
+        <v>2.230000000000001</v>
       </c>
       <c r="B129" t="n">
-        <v>0.3018772381773177</v>
+        <v>0.3003465771522537</v>
       </c>
       <c r="C129" t="n">
-        <v>0.3089497592696021</v>
+        <v>0.3140079725400088</v>
       </c>
       <c r="D129" t="n">
-        <v>0.5246000000000001</v>
+        <v>0.5254</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>2.280000000000001</v>
+        <v>2.240000000000001</v>
       </c>
       <c r="B130" t="n">
-        <v>0.3024471741852424</v>
+        <v>0.3006155829702431</v>
       </c>
       <c r="C130" t="n">
-        <v>0.3079377243999089</v>
+        <v>0.3125840059008641</v>
       </c>
       <c r="D130" t="n">
-        <v>0.5244</v>
+        <v>0.5252</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>2.290000000000001</v>
+        <v>2.250000000000001</v>
       </c>
       <c r="B131" t="n">
-        <v>0.3030904332038758</v>
+        <v>0.3009607359798385</v>
       </c>
       <c r="C131" t="n">
-        <v>0.3070176375823833</v>
+        <v>0.3112686736736835</v>
       </c>
       <c r="D131" t="n">
-        <v>0.5242</v>
+        <v>0.525</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>2.300000000000001</v>
+        <v>2.260000000000001</v>
       </c>
       <c r="B132" t="n">
-        <v>0.3038060233744357</v>
+        <v>0.3013815039801162</v>
       </c>
       <c r="C132" t="n">
-        <v>0.3061843792354639</v>
+        <v>0.3100585863675541</v>
       </c>
       <c r="D132" t="n">
-        <v>0.524</v>
+        <v>0.5248</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>2.310000000000001</v>
+        <v>2.270000000000001</v>
       </c>
       <c r="B133" t="n">
-        <v>0.304592841308746</v>
+        <v>0.3018772381773177</v>
       </c>
       <c r="C133" t="n">
-        <v>0.3054326477742966</v>
+        <v>0.3089497592696021</v>
       </c>
       <c r="D133" t="n">
-        <v>0.5238</v>
+        <v>0.5246000000000001</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>2.320000000000001</v>
+        <v>2.280000000000001</v>
       </c>
       <c r="B134" t="n">
-        <v>0.3054496737905817</v>
+        <v>0.3024471741852424</v>
       </c>
       <c r="C134" t="n">
-        <v>0.3047570447979442</v>
+        <v>0.3079377243999089</v>
       </c>
       <c r="D134" t="n">
-        <v>0.5236000000000001</v>
+        <v>0.5244</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>2.330000000000001</v>
+        <v>2.290000000000001</v>
       </c>
       <c r="B135" t="n">
-        <v>0.3063751996463602</v>
+        <v>0.3030904332038758</v>
       </c>
       <c r="C135" t="n">
-        <v>0.3041521515043044</v>
+        <v>0.3070176375823833</v>
       </c>
       <c r="D135" t="n">
-        <v>0.5234</v>
+        <v>0.5242</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>2.340000000000001</v>
+        <v>2.300000000000001</v>
       </c>
       <c r="B136" t="n">
-        <v>0.3073679917822955</v>
+        <v>0.3038060233744357</v>
       </c>
       <c r="C136" t="n">
-        <v>0.3036125960259888</v>
+        <v>0.3061843792354639</v>
       </c>
       <c r="D136" t="n">
-        <v>0.5232</v>
+        <v>0.524</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>2.350000000000001</v>
+        <v>2.310000000000001</v>
       </c>
       <c r="B137" t="n">
-        <v>0.3084265193848729</v>
+        <v>0.304592841308746</v>
       </c>
       <c r="C137" t="n">
-        <v>0.3031331116079189</v>
+        <v>0.3054326477742966</v>
       </c>
       <c r="D137" t="n">
-        <v>0.523</v>
+        <v>0.5238</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>2.360000000000001</v>
+        <v>2.320000000000001</v>
       </c>
       <c r="B138" t="n">
-        <v>0.3095491502812527</v>
+        <v>0.3054496737905817</v>
       </c>
       <c r="C138" t="n">
-        <v>0.3027085857485618</v>
+        <v>0.3047570447979442</v>
       </c>
       <c r="D138" t="n">
-        <v>0.5228</v>
+        <v>0.5236000000000001</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>2.370000000000001</v>
+        <v>2.330000000000001</v>
       </c>
       <c r="B139" t="n">
-        <v>0.3107341534559628</v>
+        <v>0.3063751996463602</v>
       </c>
       <c r="C139" t="n">
-        <v>0.3023341005994573</v>
+        <v>0.3041521515043044</v>
       </c>
       <c r="D139" t="n">
-        <v>0.5226000000000001</v>
+        <v>0.5234</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>2.380000000000001</v>
+        <v>2.340000000000001</v>
       </c>
       <c r="B140" t="n">
-        <v>0.3119797017199986</v>
+        <v>0.3073679917822955</v>
       </c>
       <c r="C140" t="n">
-        <v>0.3020049650610047</v>
+        <v>0.3036125960259888</v>
       </c>
       <c r="D140" t="n">
-        <v>0.5224</v>
+        <v>0.5232</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>2.390000000000001</v>
+        <v>2.350000000000001</v>
       </c>
       <c r="B141" t="n">
-        <v>0.3132838745282159</v>
+        <v>0.3084265193848729</v>
       </c>
       <c r="C141" t="n">
-        <v>0.3017167391264064</v>
+        <v>0.3031331116079189</v>
       </c>
       <c r="D141" t="n">
-        <v>0.5222</v>
+        <v>0.523</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>2.400000000000001</v>
+        <v>2.360000000000001</v>
       </c>
       <c r="B142" t="n">
-        <v>0.3146446609406727</v>
+        <v>0.3095491502812527</v>
       </c>
       <c r="C142" t="n">
-        <v>0.3014652511110987</v>
+        <v>0.3027085857485618</v>
       </c>
       <c r="D142" t="n">
-        <v>0.522</v>
+        <v>0.5228</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>2.410000000000001</v>
+        <v>2.370000000000001</v>
       </c>
       <c r="B143" t="n">
-        <v>0.316059962723353</v>
+        <v>0.3107341534559628</v>
       </c>
       <c r="C143" t="n">
-        <v>0.3012466084635467</v>
+        <v>0.3023341005994573</v>
       </c>
       <c r="D143" t="n">
-        <v>0.5218</v>
+        <v>0.5226000000000001</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>2.420000000000001</v>
+        <v>2.380000000000001</v>
       </c>
       <c r="B144" t="n">
-        <v>0.317527597583491</v>
+        <v>0.3119797017199986</v>
       </c>
       <c r="C144" t="n">
-        <v>0.3010572028871388</v>
+        <v>0.3020049650610047</v>
       </c>
       <c r="D144" t="n">
-        <v>0.5216000000000001</v>
+        <v>0.5224</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>2.430000000000001</v>
+        <v>2.390000000000001</v>
       </c>
       <c r="B145" t="n">
-        <v>0.3190453025345085</v>
+        <v>0.3132838745282159</v>
       </c>
       <c r="C145" t="n">
-        <v>0.3008937105146824</v>
+        <v>0.3017167391264064</v>
       </c>
       <c r="D145" t="n">
-        <v>0.5214</v>
+        <v>0.5222</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>2.440000000000001</v>
+        <v>2.400000000000001</v>
       </c>
       <c r="B146" t="n">
-        <v>0.3206107373853765</v>
+        <v>0.3146446609406727</v>
       </c>
       <c r="C146" t="n">
-        <v>0.3007530878695761</v>
+        <v>0.3014652511110987</v>
       </c>
       <c r="D146" t="n">
-        <v>0.5212</v>
+        <v>0.522</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>2.450000000000001</v>
+        <v>2.410000000000001</v>
       </c>
       <c r="B147" t="n">
-        <v>0.32222148834902</v>
+        <v>0.316059962723353</v>
       </c>
       <c r="C147" t="n">
-        <v>0.3006325643241274</v>
+        <v>0.3012466084635467</v>
       </c>
       <c r="D147" t="n">
-        <v>0.521</v>
+        <v>0.5218</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>2.460000000000001</v>
+        <v>2.420000000000001</v>
       </c>
       <c r="B148" t="n">
-        <v>0.3238750717642027</v>
+        <v>0.317527597583491</v>
       </c>
       <c r="C148" t="n">
-        <v>0.3005296317287744</v>
+        <v>0.3010572028871388</v>
       </c>
       <c r="D148" t="n">
-        <v>0.5208</v>
+        <v>0.5216000000000001</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>2.470000000000002</v>
+        <v>2.430000000000001</v>
       </c>
       <c r="B149" t="n">
-        <v>0.3255689379251525</v>
+        <v>0.3190453025345085</v>
       </c>
       <c r="C149" t="n">
-        <v>0.3004420318391043</v>
+        <v>0.3008937105146824</v>
       </c>
       <c r="D149" t="n">
-        <v>0.5206000000000001</v>
+        <v>0.5214</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>2.480000000000001</v>
+        <v>2.440000000000001</v>
       </c>
       <c r="B150" t="n">
-        <v>0.3273004750130228</v>
+        <v>0.3206107373853765</v>
       </c>
       <c r="C150" t="n">
-        <v>0.3003677421133822</v>
+        <v>0.3007530878695761</v>
       </c>
       <c r="D150" t="n">
-        <v>0.5204</v>
+        <v>0.5212</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>2.490000000000001</v>
+        <v>2.450000000000001</v>
       </c>
       <c r="B151" t="n">
-        <v>0.3290670131231287</v>
+        <v>0.32222148834902</v>
       </c>
       <c r="C151" t="n">
-        <v>0.3003049603943715</v>
+        <v>0.3006325643241274</v>
       </c>
       <c r="D151" t="n">
-        <v>0.5202</v>
+        <v>0.521</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>2.500000000000001</v>
+        <v>2.460000000000001</v>
       </c>
       <c r="B152" t="n">
-        <v>0.3308658283817457</v>
+        <v>0.3238750717642027</v>
       </c>
       <c r="C152" t="n">
-        <v>0.3002520889278755</v>
+        <v>0.3005296317287744</v>
       </c>
       <c r="D152" t="n">
-        <v>0.52</v>
+        <v>0.5208</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>2.510000000000002</v>
+        <v>2.470000000000002</v>
       </c>
       <c r="B153" t="n">
-        <v>0.3326941471461256</v>
+        <v>0.3255689379251525</v>
       </c>
       <c r="C153" t="n">
-        <v>0.3002077181086515</v>
+        <v>0.3004420318391043</v>
       </c>
       <c r="D153" t="n">
-        <v>0.5198</v>
+        <v>0.5206000000000001</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>2.520000000000001</v>
+        <v>2.480000000000001</v>
       </c>
       <c r="B154" t="n">
-        <v>0.3345491502812528</v>
+        <v>0.3273004750130228</v>
       </c>
       <c r="C154" t="n">
-        <v>0.3001706102838388</v>
+        <v>0.3003677421133822</v>
       </c>
       <c r="D154" t="n">
-        <v>0.5196000000000001</v>
+        <v>0.5204</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>2.530000000000001</v>
+        <v>2.490000000000001</v>
       </c>
       <c r="B155" t="n">
-        <v>0.3364279775067465</v>
+        <v>0.3290670131231287</v>
       </c>
       <c r="C155" t="n">
-        <v>0.3001396838861702</v>
+        <v>0.3003049603943715</v>
       </c>
       <c r="D155" t="n">
-        <v>0.5194</v>
+        <v>0.5202</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>2.540000000000001</v>
+        <v>2.500000000000001</v>
       </c>
       <c r="B156" t="n">
-        <v>0.338327731807205</v>
+        <v>0.3308658283817457</v>
       </c>
       <c r="C156" t="n">
-        <v>0.3001139981150554</v>
+        <v>0.3002520889278755</v>
       </c>
       <c r="D156" t="n">
-        <v>0.5192</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>2.550000000000002</v>
+        <v>2.510000000000002</v>
       </c>
       <c r="B157" t="n">
-        <v>0.3402454838991938</v>
+        <v>0.3326941471461256</v>
       </c>
       <c r="C157" t="n">
-        <v>0.3000927383339124</v>
+        <v>0.3002077181086515</v>
       </c>
       <c r="D157" t="n">
-        <v>0.519</v>
+        <v>0.5198</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>2.560000000000001</v>
+        <v>2.520000000000001</v>
       </c>
       <c r="B158" t="n">
-        <v>0.3421782767479887</v>
+        <v>0.3345491502812528</v>
       </c>
       <c r="C158" t="n">
-        <v>0.3000752023073744</v>
+        <v>0.3001706102838388</v>
       </c>
       <c r="D158" t="n">
-        <v>0.5188</v>
+        <v>0.5196000000000001</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>2.570000000000001</v>
+        <v>2.530000000000001</v>
       </c>
       <c r="B159" t="n">
-        <v>0.3441231301271083</v>
+        <v>0.3364279775067465</v>
       </c>
       <c r="C159" t="n">
-        <v>0.3000607873624943</v>
+        <v>0.3001396838861702</v>
       </c>
       <c r="D159" t="n">
-        <v>0.5186000000000001</v>
+        <v>0.5194</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>2.580000000000001</v>
+        <v>2.540000000000001</v>
       </c>
       <c r="B160" t="n">
-        <v>0.346077045213608</v>
+        <v>0.338327731807205</v>
       </c>
       <c r="C160" t="n">
-        <v>0.3000489785238695</v>
+        <v>0.3001139981150554</v>
       </c>
       <c r="D160" t="n">
-        <v>0.5184</v>
+        <v>0.5192</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>2.590000000000002</v>
+        <v>2.550000000000002</v>
       </c>
       <c r="B161" t="n">
-        <v>0.3480370092120469</v>
+        <v>0.3402454838991938</v>
       </c>
       <c r="C161" t="n">
-        <v>0.3000393376436319</v>
+        <v>0.3000927383339124</v>
       </c>
       <c r="D161" t="n">
-        <v>0.5182</v>
+        <v>0.519</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
+        <v>2.560000000000001</v>
+      </c>
+      <c r="B162" t="n">
+        <v>0.3421782767479887</v>
+      </c>
+      <c r="C162" t="n">
+        <v>0.3000752023073744</v>
+      </c>
+      <c r="D162" t="n">
+        <v>0.5188</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>2.570000000000001</v>
+      </c>
+      <c r="B163" t="n">
+        <v>0.3441231301271083</v>
+      </c>
+      <c r="C163" t="n">
+        <v>0.3000607873624943</v>
+      </c>
+      <c r="D163" t="n">
+        <v>0.5186000000000001</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>2.580000000000001</v>
+      </c>
+      <c r="B164" t="n">
+        <v>0.346077045213608</v>
+      </c>
+      <c r="C164" t="n">
+        <v>0.3000489785238695</v>
+      </c>
+      <c r="D164" t="n">
+        <v>0.5184</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>2.590000000000002</v>
+      </c>
+      <c r="B165" t="n">
+        <v>0.3480370092120469</v>
+      </c>
+      <c r="C165" t="n">
+        <v>0.3000393376436319</v>
+      </c>
+      <c r="D165" t="n">
+        <v>0.5182</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
         <v>2.600000000000001</v>
       </c>
-      <c r="B162" t="n">
+      <c r="B166" t="n">
         <v>0.3500000000000003</v>
       </c>
-      <c r="C162" t="n">
+      <c r="C166" t="n">
         <v>0.3000314935232524</v>
       </c>
-      <c r="D162" t="n">
+      <c r="D166" t="n">
         <v>0.518</v>
       </c>
     </row>

</xml_diff>